<commit_message>
Add new street, unit abbreviations to .xlsx files.
</commit_message>
<xml_diff>
--- a/src/redcaputilities/data/unit_abbreviations.xlsx
+++ b/src/redcaputilities/data/unit_abbreviations.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GitHub\REDCapMatchResolver\src\redcapmatchresolver\data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GitHub\REDCapUtilities\src\redcaputilities\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{D7E7FABA-AB37-4AF3-A837-D340A9780B2B}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C33CDB3A-E7B4-446D-B815-0B953640A34E}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="21570" windowHeight="7980" xr2:uid="{3F1AA00E-824F-45E6-8A29-50C9C1A1E684}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="22">
   <si>
     <t>Unit designator</t>
   </si>
@@ -70,6 +70,27 @@
   </si>
   <si>
     <t>DEPT</t>
+  </si>
+  <si>
+    <t>HANGAR</t>
+  </si>
+  <si>
+    <t>HNGR</t>
+  </si>
+  <si>
+    <t>LOT</t>
+  </si>
+  <si>
+    <t>SPACE</t>
+  </si>
+  <si>
+    <t>SPC</t>
+  </si>
+  <si>
+    <t>NUMBER</t>
+  </si>
+  <si>
+    <t>BLD</t>
   </si>
 </sst>
 </file>
@@ -468,7 +489,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2ECA580C-9AB0-4DA0-BF28-58C56BEB2556}">
-  <dimension ref="A1:B8"/>
+  <dimension ref="A1:B13"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="14.7109375" bestFit="1" customWidth="1"/>
@@ -493,7 +514,7 @@
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
-        <v>4</v>
+        <v>21</v>
       </c>
       <c r="B3" s="2" t="s">
         <v>5</v>
@@ -501,42 +522,82 @@
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>9</v>
+        <v>14</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>12</v>
+        <v>16</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>14</v>
+        <v>17</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A9" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A10" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A11" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A12" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A13" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>10</v>
       </c>
     </row>
   </sheetData>

</xml_diff>